<commit_message>
Listener concept with Retry Analyzer
</commit_message>
<xml_diff>
--- a/testData/loginData.xlsx
+++ b/testData/loginData.xlsx
@@ -27,13 +27,13 @@
     <t>loginVerify</t>
   </si>
   <si>
-    <t>standard_user</t>
-  </si>
-  <si>
-    <t>secret_sauce</t>
-  </si>
-  <si>
-    <t>Swag Labs</t>
+    <t>mail_2_logeshwaran@gmail.com</t>
+  </si>
+  <si>
+    <t>N@th@niel01-26</t>
+  </si>
+  <si>
+    <t>My Account</t>
   </si>
 </sst>
 </file>
@@ -375,9 +375,9 @@
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>